<commit_message>
finalized code pre-optimization and cleanup
</commit_message>
<xml_diff>
--- a/code/dependencies/regionCategories.xlsx
+++ b/code/dependencies/regionCategories.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Samsung_T5/cingulateConnectivity/code/dependencies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B121F5E9-358E-154E-B0B1-79D4F8FE6EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61EAD9D3-D992-0B49-908F-69C3A3C7BBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51140" yWindow="2120" windowWidth="28040" windowHeight="27180" xr2:uid="{412C4C44-F877-F24A-A26F-D981E192A21E}"/>
+    <workbookView xWindow="-13600" yWindow="500" windowWidth="13600" windowHeight="14860" xr2:uid="{412C4C44-F877-F24A-A26F-D981E192A21E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="217">
   <si>
     <t>G_and_S_frontomargin</t>
   </si>
@@ -1261,6 +1261,69 @@
   </si>
   <si>
     <t>Hippocampus</t>
+  </si>
+  <si>
+    <t>Accessory Basal Nucleus of the Amygdala</t>
+  </si>
+  <si>
+    <t>Anterior Amygdaloid Area</t>
+  </si>
+  <si>
+    <t>Basal Nucleus of the Amygdala</t>
+  </si>
+  <si>
+    <t>Body of the Cornu Ammonis Area 1</t>
+  </si>
+  <si>
+    <t>Head of the Cornu Ammonis Area 1</t>
+  </si>
+  <si>
+    <t>Head of the Cornu Ammonis Area 3</t>
+  </si>
+  <si>
+    <t>Body of the polymorphic layer of the dentate gyrus</t>
+  </si>
+  <si>
+    <t>Head of the polymorphic layer of the dentate gyrus</t>
+  </si>
+  <si>
+    <t>Corticoamygdaloid transition area</t>
+  </si>
+  <si>
+    <t>The Temporal pole</t>
+  </si>
+  <si>
+    <t>Body of the granule cell and molecular layer of the dentate gyrus</t>
+  </si>
+  <si>
+    <t>Head of the granule cell and molecular layer of the dentate gyrus</t>
+  </si>
+  <si>
+    <t>Hippocampal-amygdaloid transition area</t>
+  </si>
+  <si>
+    <t>Hippocampal Fissure</t>
+  </si>
+  <si>
+    <t>Body of the molecular layer of the hippocampus</t>
+  </si>
+  <si>
+    <t>Head of the molecular layer of the hippocampus</t>
+  </si>
+  <si>
+    <t>Body of the presubiculum</t>
+  </si>
+  <si>
+    <t>Body of the subiculum</t>
+  </si>
+  <si>
+    <t>Head of the subiculum</t>
+  </si>
+  <si>
+    <t>Lateral nucleus of the amygdala</t>
+  </si>
+  <si>
+    <t>Paralaminar nucleus of the amygdala</t>
   </si>
 </sst>
 </file>
@@ -1672,14 +1735,14 @@
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>196</v>
       </c>
       <c r="C2" t="s">
-        <v>151</v>
+        <v>185</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1688,14 +1751,14 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
+      <c r="A3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>197</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>185</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1704,14 +1767,14 @@
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
+      <c r="A4" t="s">
+        <v>164</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>5</v>
+        <v>198</v>
       </c>
       <c r="C4" t="s">
-        <v>153</v>
+        <v>185</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1720,14 +1783,14 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
+      <c r="A5" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>204</v>
       </c>
       <c r="C5" t="s">
-        <v>152</v>
+        <v>185</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -1736,14 +1799,14 @@
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>9</v>
+      <c r="A6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>215</v>
       </c>
       <c r="C6" t="s">
-        <v>151</v>
+        <v>185</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1752,14 +1815,14 @@
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>11</v>
+      <c r="A7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="C7" t="s">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1769,10 +1832,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
         <v>155</v>
@@ -1785,10 +1848,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
         <v>155</v>
@@ -1801,10 +1864,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
         <v>155</v>
@@ -1817,10 +1880,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
         <v>155</v>
@@ -1833,13 +1896,13 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -1849,13 +1912,13 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -1865,10 +1928,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>25</v>
+        <v>0</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C14" t="s">
         <v>151</v>
@@ -1881,10 +1944,10 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>27</v>
+        <v>8</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="C15" t="s">
         <v>151</v>
@@ -1897,10 +1960,10 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C16" t="s">
         <v>151</v>
@@ -1913,10 +1976,10 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
         <v>151</v>
@@ -1929,13 +1992,13 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C18" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1945,13 +2008,13 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1961,13 +2024,13 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>37</v>
+        <v>30</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="C20" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1977,13 +2040,13 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>39</v>
+        <v>102</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -1993,13 +2056,13 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>41</v>
+        <v>104</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="C22" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -2009,13 +2072,13 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="C23" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -2024,14 +2087,14 @@
       <c r="H23" s="1"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
-        <v>44</v>
+      <c r="A24" t="s">
+        <v>165</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>45</v>
+        <v>199</v>
       </c>
       <c r="C24" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -2040,14 +2103,14 @@
       <c r="H24" s="1"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
-        <v>46</v>
+      <c r="A25" t="s">
+        <v>166</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="C25" t="s">
-        <v>158</v>
+        <v>195</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -2056,14 +2119,14 @@
       <c r="H25" s="1"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
-        <v>48</v>
+      <c r="A26" t="s">
+        <v>167</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>49</v>
+        <v>201</v>
       </c>
       <c r="C26" t="s">
-        <v>153</v>
+        <v>195</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -2072,14 +2135,14 @@
       <c r="H26" s="1"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>50</v>
+      <c r="A27" t="s">
+        <v>168</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>51</v>
+        <v>202</v>
       </c>
       <c r="C27" t="s">
-        <v>153</v>
+        <v>195</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -2088,14 +2151,14 @@
       <c r="H27" s="1"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="1" t="s">
-        <v>52</v>
+      <c r="A28" t="s">
+        <v>169</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>53</v>
+        <v>203</v>
       </c>
       <c r="C28" t="s">
-        <v>153</v>
+        <v>195</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
@@ -2104,14 +2167,14 @@
       <c r="H28" s="1"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
-        <v>54</v>
+      <c r="A29" t="s">
+        <v>171</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>55</v>
+        <v>206</v>
       </c>
       <c r="C29" t="s">
-        <v>159</v>
+        <v>195</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
@@ -2120,14 +2183,14 @@
       <c r="H29" s="1"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
-        <v>56</v>
+      <c r="A30" t="s">
+        <v>172</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>57</v>
+        <v>207</v>
       </c>
       <c r="C30" t="s">
-        <v>160</v>
+        <v>195</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
@@ -2136,14 +2199,14 @@
       <c r="H30" s="1"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
-        <v>58</v>
+      <c r="A31" t="s">
+        <v>173</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>59</v>
+        <v>208</v>
       </c>
       <c r="C31" t="s">
-        <v>153</v>
+        <v>195</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
@@ -2152,14 +2215,14 @@
       <c r="H31" s="1"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
-        <v>60</v>
+      <c r="A32" t="s">
+        <v>178</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>61</v>
+        <v>209</v>
       </c>
       <c r="C32" t="s">
-        <v>158</v>
+        <v>195</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -2168,14 +2231,14 @@
       <c r="H32" s="1"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
-        <v>62</v>
+      <c r="A33" t="s">
+        <v>179</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>63</v>
+        <v>210</v>
       </c>
       <c r="C33" t="s">
-        <v>161</v>
+        <v>195</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -2184,14 +2247,14 @@
       <c r="H33" s="1"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
-        <v>64</v>
+      <c r="A34" t="s">
+        <v>180</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>65</v>
+        <v>211</v>
       </c>
       <c r="C34" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
@@ -2200,14 +2263,14 @@
       <c r="H34" s="1"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>67</v>
+      <c r="A35" t="s">
+        <v>181</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>212</v>
       </c>
       <c r="C35" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -2216,14 +2279,14 @@
       <c r="H35" s="1"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>69</v>
+      <c r="A36" t="s">
+        <v>182</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>213</v>
       </c>
       <c r="C36" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
@@ -2232,14 +2295,14 @@
       <c r="H36" s="1"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
-        <v>70</v>
+      <c r="A37" t="s">
+        <v>183</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>71</v>
+        <v>214</v>
       </c>
       <c r="C37" t="s">
-        <v>157</v>
+        <v>195</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -2249,13 +2312,13 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="C38" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
@@ -2265,13 +2328,13 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>74</v>
+        <v>34</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="C39" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
@@ -2281,13 +2344,13 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="C40" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
@@ -2297,13 +2360,13 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="C41" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
@@ -2313,13 +2376,13 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>81</v>
+        <v>96</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="C42" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
@@ -2329,13 +2392,13 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="C43" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
@@ -2345,13 +2408,13 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>85</v>
+        <v>134</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>135</v>
       </c>
       <c r="C44" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
@@ -2361,13 +2424,13 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>87</v>
+        <v>136</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>137</v>
       </c>
       <c r="C45" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
@@ -2377,13 +2440,13 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>89</v>
+        <v>2</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="C46" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
@@ -2393,13 +2456,13 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>91</v>
+        <v>21</v>
       </c>
       <c r="C47" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
@@ -2409,13 +2472,13 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>92</v>
+        <v>36</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>93</v>
+        <v>37</v>
       </c>
       <c r="C48" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
@@ -2425,13 +2488,13 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="C49" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
@@ -2441,13 +2504,13 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>97</v>
+        <v>82</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>83</v>
       </c>
       <c r="C50" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
@@ -2457,13 +2520,13 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>99</v>
+        <v>86</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="C51" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
@@ -2489,13 +2552,13 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>103</v>
+        <v>112</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="C53" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
@@ -2505,13 +2568,13 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="C54" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
@@ -2521,13 +2584,13 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>107</v>
+        <v>116</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="C55" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
@@ -2537,13 +2600,13 @@
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>109</v>
+        <v>128</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>129</v>
       </c>
       <c r="C56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
@@ -2553,13 +2616,13 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>111</v>
+        <v>6</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C57" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
@@ -2569,13 +2632,13 @@
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>112</v>
+        <v>76</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="C58" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
@@ -2585,13 +2648,13 @@
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="C59" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
@@ -2601,13 +2664,13 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>117</v>
+        <v>80</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="C60" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D60" s="1"/>
       <c r="E60" s="1"/>
@@ -2617,13 +2680,13 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>119</v>
+        <v>46</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="C61" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D61" s="1"/>
       <c r="E61" s="1"/>
@@ -2633,13 +2696,13 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>121</v>
+        <v>60</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="C62" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D62" s="1"/>
       <c r="E62" s="1"/>
@@ -2697,13 +2760,13 @@
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>129</v>
+        <v>138</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>139</v>
       </c>
       <c r="C66" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D66" s="1"/>
       <c r="E66" s="1"/>
@@ -2713,10 +2776,10 @@
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>131</v>
+        <v>62</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="C67" t="s">
         <v>161</v>
@@ -2729,13 +2792,13 @@
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="C68" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D68" s="1"/>
       <c r="E68" s="1"/>
@@ -2744,14 +2807,11 @@
       <c r="H68" s="1"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>135</v>
+      <c r="A69" t="s">
+        <v>191</v>
       </c>
       <c r="C69" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D69" s="1"/>
       <c r="E69" s="1"/>
@@ -2760,14 +2820,11 @@
       <c r="H69" s="1"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>137</v>
+      <c r="A70" t="s">
+        <v>187</v>
       </c>
       <c r="C70" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D70" s="1"/>
       <c r="E70" s="1"/>
@@ -2776,14 +2833,11 @@
       <c r="H70" s="1"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>139</v>
+      <c r="A71" t="s">
+        <v>192</v>
       </c>
       <c r="C71" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D71" s="1"/>
       <c r="E71" s="1"/>
@@ -2792,14 +2846,11 @@
       <c r="H71" s="1"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A72" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>141</v>
+      <c r="A72" t="s">
+        <v>188</v>
       </c>
       <c r="C72" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="D72" s="1"/>
       <c r="E72" s="1"/>
@@ -2808,14 +2859,11 @@
       <c r="H72" s="1"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A73" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>143</v>
+      <c r="A73" t="s">
+        <v>189</v>
       </c>
       <c r="C73" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D73" s="1"/>
       <c r="E73" s="1"/>
@@ -2824,14 +2872,11 @@
       <c r="H73" s="1"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A74" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>145</v>
+      <c r="A74" t="s">
+        <v>193</v>
       </c>
       <c r="C74" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D74" s="1"/>
       <c r="E74" s="1"/>
@@ -2840,273 +2885,360 @@
       <c r="H74" s="1"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A75" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>147</v>
+      <c r="A75" t="s">
+        <v>176</v>
       </c>
       <c r="C75" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
       <c r="C76" t="s">
-        <v>185</v>
+        <v>161</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>163</v>
+      <c r="A77" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C77" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>164</v>
+      <c r="A78" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="C78" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>165</v>
+      <c r="A79" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>51</v>
       </c>
       <c r="C79" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>166</v>
+      <c r="A80" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="C80" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>167</v>
+      <c r="A81" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="C81" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>168</v>
+      <c r="A82" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>109</v>
       </c>
       <c r="C82" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>169</v>
+      <c r="A83" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="C83" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>170</v>
+      <c r="A84" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="C84" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>171</v>
+      <c r="A85" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="C85" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>172</v>
+      <c r="A86" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>89</v>
       </c>
       <c r="C86" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>173</v>
+      <c r="A87" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>133</v>
       </c>
       <c r="C87" t="s">
-        <v>195</v>
+        <v>159</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>174</v>
+      <c r="A88" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="C88" t="s">
-        <v>185</v>
+        <v>157</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>175</v>
+      <c r="A89" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="C89" t="s">
-        <v>185</v>
+        <v>157</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>84</v>
+      <c r="A90" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="C90" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>191</v>
+      <c r="A91" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="C91" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>186</v>
+      <c r="A92" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="C92" t="s">
-        <v>194</v>
+        <v>157</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>187</v>
+      <c r="A93" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>69</v>
       </c>
       <c r="C93" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>192</v>
+      <c r="A94" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>71</v>
       </c>
       <c r="C94" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>188</v>
+      <c r="A95" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="C95" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>189</v>
+      <c r="A96" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="C96" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>190</v>
+      <c r="A97" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>85</v>
       </c>
       <c r="C97" t="s">
-        <v>190</v>
+        <v>157</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>193</v>
+      <c r="A98" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="C98" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>176</v>
+      <c r="A99" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>119</v>
       </c>
       <c r="C99" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
-        <v>177</v>
+      <c r="A100" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="C100" t="s">
-        <v>194</v>
+        <v>157</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>178</v>
+      <c r="A101" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>143</v>
       </c>
       <c r="C101" t="s">
-        <v>195</v>
+        <v>157</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>179</v>
+      <c r="A102" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>145</v>
       </c>
       <c r="C102" t="s">
-        <v>195</v>
+        <v>157</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>180</v>
+      <c r="A103" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>147</v>
       </c>
       <c r="C103" t="s">
-        <v>195</v>
+        <v>157</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>181</v>
+        <v>84</v>
+      </c>
+      <c r="B104" t="s">
+        <v>205</v>
       </c>
       <c r="C104" t="s">
-        <v>195</v>
+        <v>157</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>182</v>
+        <v>190</v>
+      </c>
+      <c r="B105" t="s">
+        <v>190</v>
       </c>
       <c r="C105" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C106" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="C107" t="s">
-        <v>161</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C107">
+    <sortCondition ref="C2:C107"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>